<commit_message>
Inclusão da coluna classificacao
</commit_message>
<xml_diff>
--- a/DEMANDAS_DOWNSTREAM_V3.xlsx
+++ b/DEMANDAS_DOWNSTREAM_V3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\PROFISSIONAL\ANP\APRESENTACAO_IA_MAIO_2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gsc\Desktop\ML_DEMANDAS_TI\machine-learning-demandas-ti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E2D563-838F-4504-AB55-841F16A6EABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{251A0EC7-CE62-42B8-9B05-DC8CDF0B588D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2059,7 +2059,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2067,12 +2067,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2088,10 +2082,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7750,41 +7740,41 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="141" spans="1:12" s="6" customFormat="1">
-      <c r="A141" s="5">
+    <row r="141" spans="1:12">
+      <c r="A141" s="1">
         <v>21626</v>
       </c>
-      <c r="B141" s="6" t="s">
+      <c r="B141" t="s">
         <v>14</v>
       </c>
-      <c r="C141" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D141" s="6" t="s">
+      <c r="C141" t="s">
+        <v>12</v>
+      </c>
+      <c r="D141" t="s">
         <v>9</v>
       </c>
-      <c r="E141" s="5">
+      <c r="E141" s="1">
         <v>32</v>
       </c>
-      <c r="F141" s="5">
+      <c r="F141" s="1">
         <v>2026</v>
       </c>
-      <c r="G141" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H141" s="7">
+      <c r="G141" t="s">
+        <v>10</v>
+      </c>
+      <c r="H141" s="2">
         <v>46029.751574074071</v>
       </c>
-      <c r="I141" s="7">
+      <c r="I141" s="2">
         <v>46031.567766203705</v>
       </c>
-      <c r="J141" s="7">
+      <c r="J141" s="2">
         <v>46031.909780092596</v>
       </c>
-      <c r="K141" s="8" t="s">
+      <c r="K141" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="L141" s="7">
+      <c r="L141" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -9194,41 +9184,41 @@
         <v>46010</v>
       </c>
     </row>
-    <row r="179" spans="1:12" s="6" customFormat="1">
-      <c r="A179" s="5">
+    <row r="179" spans="1:12">
+      <c r="A179" s="1">
         <v>21491</v>
       </c>
-      <c r="B179" s="6" t="s">
+      <c r="B179" t="s">
         <v>14</v>
       </c>
-      <c r="C179" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D179" s="6" t="s">
+      <c r="C179" t="s">
+        <v>12</v>
+      </c>
+      <c r="D179" t="s">
         <v>13</v>
       </c>
-      <c r="E179" s="5">
+      <c r="E179" s="1">
         <v>2403</v>
       </c>
-      <c r="F179" s="5">
+      <c r="F179" s="1">
         <v>2025</v>
       </c>
-      <c r="G179" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H179" s="7">
+      <c r="G179" t="s">
+        <v>10</v>
+      </c>
+      <c r="H179" s="2">
         <v>46000.66746527778</v>
       </c>
-      <c r="I179" s="7">
+      <c r="I179" s="2">
         <v>46001.451921296299</v>
       </c>
-      <c r="J179" s="7">
+      <c r="J179" s="2">
         <v>46001.511944444443</v>
       </c>
-      <c r="K179" s="8" t="s">
+      <c r="K179" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="L179" s="7">
+      <c r="L179" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -10790,41 +10780,41 @@
         <v>45985</v>
       </c>
     </row>
-    <row r="221" spans="1:12" s="6" customFormat="1">
-      <c r="A221" s="5">
+    <row r="221" spans="1:12">
+      <c r="A221" s="1">
         <v>21376</v>
       </c>
-      <c r="B221" s="6" t="s">
+      <c r="B221" t="s">
         <v>19</v>
       </c>
-      <c r="C221" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D221" s="6" t="s">
+      <c r="C221" t="s">
+        <v>12</v>
+      </c>
+      <c r="D221" t="s">
         <v>15</v>
       </c>
-      <c r="E221" s="5">
+      <c r="E221" s="1">
         <v>2288</v>
       </c>
-      <c r="F221" s="5">
+      <c r="F221" s="1">
         <v>2025</v>
       </c>
-      <c r="G221" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H221" s="7">
+      <c r="G221" t="s">
+        <v>10</v>
+      </c>
+      <c r="H221" s="2">
         <v>45979.708425925928</v>
       </c>
-      <c r="I221" s="7">
+      <c r="I221" s="2">
         <v>45986.720185185186</v>
       </c>
-      <c r="J221" s="7">
+      <c r="J221" s="2">
         <v>45986.762314814812</v>
       </c>
-      <c r="K221" s="8" t="s">
+      <c r="K221" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="L221" s="7">
+      <c r="L221" s="2">
         <v>45987</v>
       </c>
     </row>
@@ -11322,41 +11312,41 @@
         <v>45972</v>
       </c>
     </row>
-    <row r="235" spans="1:12" s="6" customFormat="1">
-      <c r="A235" s="5">
+    <row r="235" spans="1:12">
+      <c r="A235" s="1">
         <v>21301</v>
       </c>
-      <c r="B235" s="6" t="s">
+      <c r="B235" t="s">
         <v>16</v>
       </c>
-      <c r="C235" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D235" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E235" s="5">
+      <c r="C235" t="s">
+        <v>12</v>
+      </c>
+      <c r="D235" t="s">
+        <v>17</v>
+      </c>
+      <c r="E235" s="1">
         <v>2213</v>
       </c>
-      <c r="F235" s="5">
+      <c r="F235" s="1">
         <v>2025</v>
       </c>
-      <c r="G235" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H235" s="7">
+      <c r="G235" t="s">
+        <v>10</v>
+      </c>
+      <c r="H235" s="2">
         <v>45968.378854166665</v>
       </c>
-      <c r="I235" s="7">
+      <c r="I235" s="2">
         <v>45968.40215277778</v>
       </c>
-      <c r="J235" s="7">
+      <c r="J235" s="2">
         <v>45968.416990740741</v>
       </c>
-      <c r="K235" s="8" t="s">
+      <c r="K235" s="4" t="s">
         <v>450</v>
       </c>
-      <c r="L235" s="7">
+      <c r="L235" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -11626,41 +11616,41 @@
         <v>45965</v>
       </c>
     </row>
-    <row r="243" spans="1:12" s="6" customFormat="1">
-      <c r="A243" s="5">
+    <row r="243" spans="1:12">
+      <c r="A243" s="1">
         <v>21247</v>
       </c>
-      <c r="B243" s="6" t="s">
+      <c r="B243" t="s">
         <v>19</v>
       </c>
-      <c r="C243" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D243" s="6" t="s">
+      <c r="C243" t="s">
+        <v>12</v>
+      </c>
+      <c r="D243" t="s">
         <v>20</v>
       </c>
-      <c r="E243" s="5">
+      <c r="E243" s="1">
         <v>2159</v>
       </c>
-      <c r="F243" s="5">
+      <c r="F243" s="1">
         <v>2025</v>
       </c>
-      <c r="G243" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H243" s="7">
+      <c r="G243" t="s">
+        <v>10</v>
+      </c>
+      <c r="H243" s="2">
         <v>45960.583981481483</v>
       </c>
-      <c r="I243" s="7">
+      <c r="I243" s="2">
         <v>45987.44059027778</v>
       </c>
-      <c r="J243" s="7">
+      <c r="J243" s="2">
         <v>45987.694699074076</v>
       </c>
-      <c r="K243" s="8" t="s">
+      <c r="K243" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="L243" s="7">
+      <c r="L243" s="2">
         <v>45993</v>
       </c>
     </row>

</xml_diff>